<commit_message>
Update generated Excel file
</commit_message>
<xml_diff>
--- a/dbc_signals.xlsx
+++ b/dbc_signals.xlsx
@@ -553,7 +553,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>0</v>
@@ -588,7 +588,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>

</xml_diff>